<commit_message>
update: payment updates for 4 CE students (2 exact, 2 overpay)
</commit_message>
<xml_diff>
--- a/backend/excel-files/sample_payment_updates.xlsx
+++ b/backend/excel-files/sample_payment_updates.xlsx
@@ -397,16 +397,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:F5"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="25.83203125" customWidth="1"/>
+    <col min="2" max="2" width="15.83203125" customWidth="1"/>
     <col min="3" max="3" width="15.83203125" customWidth="1"/>
     <col min="4" max="4" width="15.83203125" customWidth="1"/>
-    <col min="5" max="5" width="15.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="18.83203125" customWidth="1"/>
-    <col min="8" max="8" width="60.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="55.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -414,82 +412,104 @@
         <v>Index Number</v>
       </c>
       <c r="B1" t="str">
-        <v>Student Name</v>
+        <v>Total Amount</v>
       </c>
       <c r="C1" t="str">
-        <v>Total Amount</v>
+        <v>Amount Paid</v>
       </c>
       <c r="D1" t="str">
-        <v>Amount Paid</v>
+        <v>Academic Year</v>
       </c>
       <c r="E1" t="str">
-        <v>Academic Year</v>
+        <v>Semester</v>
       </c>
       <c r="F1" t="str">
-        <v>Semester</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Payment Method</v>
-      </c>
-      <c r="H1" t="str">
         <v>Note</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>UMaT/PG/0001/22</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Yaa Nkrumah</v>
+        <v>UMaT/PG/0003/22</v>
+      </c>
+      <c r="B2">
+        <v>8000</v>
       </c>
       <c r="C2">
-        <v>7700</v>
-      </c>
-      <c r="D2">
-        <v>1800</v>
+        <v>3000</v>
+      </c>
+      <c r="D2" t="str">
+        <v>2024/2025</v>
       </c>
       <c r="E2" t="str">
-        <v>2024/2025</v>
+        <v>First</v>
       </c>
       <c r="F2" t="str">
-        <v>Second</v>
-      </c>
-      <c r="G2" t="str">
-        <v>Bank Transfer</v>
-      </c>
-      <c r="H2" t="str">
-        <v>Payment update: Overpays by GHS 1000 on outstanding balance of GHS 800</v>
+        <v>Pays exact outstanding GHS 3,000 — fee fully cleared</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>UMaT/PG/0002/22</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Ato Owusu</v>
+        <v>UMaT/PG/0008/22</v>
+      </c>
+      <c r="B3">
+        <v>8000</v>
       </c>
       <c r="C3">
-        <v>11100</v>
-      </c>
-      <c r="D3">
-        <v>0</v>
+        <v>3000</v>
+      </c>
+      <c r="D3" t="str">
+        <v>2024/2025</v>
       </c>
       <c r="E3" t="str">
-        <v>2023/2024</v>
+        <v>First</v>
       </c>
       <c r="F3" t="str">
-        <v>Second</v>
-      </c>
-      <c r="G3" t="str">
-        <v>Bank Transfer</v>
-      </c>
-      <c r="H3" t="str">
-        <v>Payment update: Pays exact outstanding balance of GHS 0</v>
+        <v>Pays exact outstanding GHS 3,000 — fee fully cleared</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>UMaT/PG/0009/22</v>
+      </c>
+      <c r="B4">
+        <v>8000</v>
+      </c>
+      <c r="C4">
+        <v>4000</v>
+      </c>
+      <c r="D4" t="str">
+        <v>2024/2025</v>
+      </c>
+      <c r="E4" t="str">
+        <v>First</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Overpays by GHS 1,000 — creates credit balance</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>UMaT/PG/0015/22</v>
+      </c>
+      <c r="B5">
+        <v>8000</v>
+      </c>
+      <c r="C5">
+        <v>4000</v>
+      </c>
+      <c r="D5" t="str">
+        <v>2024/2025</v>
+      </c>
+      <c r="E5" t="str">
+        <v>First</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Overpays by GHS 1,000 — creates credit balance</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>